<commit_message>
Correction des URLs canoniques des fichiers de mapping ecd19cef660928e4ac185678607a2f786344cf0e
</commit_message>
<xml_diff>
--- a/fix-errors/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
+++ b/fix-errors/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
@@ -55,7 +55,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-18T08:13:43+00:00</t>
+    <t>2026-08-18T11:25:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -100,13 +100,13 @@
     <t>Target</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-advance-directive</t>
+    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/fr-lm-advance-directive|0.1.0</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-cda-directive-anticipee</t>
+    <t>https://interop.esante.gouv.fr/ig/cda/document-core/StructureDefinition/fr-cda-directive-anticipee|0.1.0</t>
   </si>
   <si>
     <t>FRLMAdvanceDirective</t>
@@ -178,7 +178,7 @@
     <t>FRCDADirectiveAnticipee.entryRelationship.observationMedia.value</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-advance-directive-document</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-advance-directive-document|0.1.0</t>
   </si>
   <si>
     <t>FRAdvanceDirectiveDocument</t>

</xml_diff>